<commit_message>
adding extreme test matrices
</commit_message>
<xml_diff>
--- a/typhoidsim/data/age_mix_contact.xlsx
+++ b/typhoidsim/data/age_mix_contact.xlsx
@@ -1,23 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kgrantz/active/typhoidsim/typhoidsim/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F7B2F1B-1F53-8041-B392-6F5BB836EFBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFBAEA59-984C-3E4E-9C87-B81C24A5157C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="760" windowWidth="33420" windowHeight="18040" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1140" yWindow="760" windowWidth="33420" windowHeight="18040" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pakistan" sheetId="1" r:id="rId1"/>
     <sheet name="Chile" sheetId="2" r:id="rId2"/>
     <sheet name="LLMIC" sheetId="3" r:id="rId3"/>
+    <sheet name="test1" sheetId="4" r:id="rId4"/>
+    <sheet name="test2" sheetId="5" r:id="rId5"/>
+    <sheet name="test3" sheetId="6" r:id="rId6"/>
+    <sheet name="test4" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -27,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="20">
   <si>
     <t>age_group</t>
   </si>
@@ -3406,4 +3410,3648 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF43759C-39B6-7149-8B7C-E662772FC59A}">
+  <dimension ref="A1:Q17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <v>3.4405470206708499</v>
+      </c>
+      <c r="C2" s="2">
+        <v>1.86488107415763</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2">
+        <v>0</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2">
+        <v>0</v>
+      </c>
+      <c r="N2" s="2">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2">
+        <v>0</v>
+      </c>
+      <c r="P2" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>2.0149296101776901</v>
+      </c>
+      <c r="C3" s="2">
+        <v>12.477572718840699</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2">
+        <v>0</v>
+      </c>
+      <c r="L3" s="2">
+        <v>0</v>
+      </c>
+      <c r="M3" s="2">
+        <v>0</v>
+      </c>
+      <c r="N3" s="2">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2">
+        <v>0</v>
+      </c>
+      <c r="P3" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2">
+        <v>0</v>
+      </c>
+      <c r="L4" s="2">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2">
+        <v>0</v>
+      </c>
+      <c r="N4" s="2">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2">
+        <v>0</v>
+      </c>
+      <c r="P4" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2">
+        <v>0</v>
+      </c>
+      <c r="L5" s="2">
+        <v>0</v>
+      </c>
+      <c r="M5" s="2">
+        <v>0</v>
+      </c>
+      <c r="N5" s="2">
+        <v>0</v>
+      </c>
+      <c r="O5" s="2">
+        <v>0</v>
+      </c>
+      <c r="P5" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2">
+        <v>0</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0</v>
+      </c>
+      <c r="I6" s="2">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2">
+        <v>0</v>
+      </c>
+      <c r="L6" s="2">
+        <v>0</v>
+      </c>
+      <c r="M6" s="2">
+        <v>0</v>
+      </c>
+      <c r="N6" s="2">
+        <v>0</v>
+      </c>
+      <c r="O6" s="2">
+        <v>0</v>
+      </c>
+      <c r="P6" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>0</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0</v>
+      </c>
+      <c r="J7" s="2">
+        <v>0</v>
+      </c>
+      <c r="K7" s="2">
+        <v>0</v>
+      </c>
+      <c r="L7" s="2">
+        <v>0</v>
+      </c>
+      <c r="M7" s="2">
+        <v>0</v>
+      </c>
+      <c r="N7" s="2">
+        <v>0</v>
+      </c>
+      <c r="O7" s="2">
+        <v>0</v>
+      </c>
+      <c r="P7" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <v>0</v>
+      </c>
+      <c r="C8" s="2">
+        <v>0</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2">
+        <v>0</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2">
+        <v>0</v>
+      </c>
+      <c r="J8" s="2">
+        <v>0</v>
+      </c>
+      <c r="K8" s="2">
+        <v>0</v>
+      </c>
+      <c r="L8" s="2">
+        <v>0</v>
+      </c>
+      <c r="M8" s="2">
+        <v>0</v>
+      </c>
+      <c r="N8" s="2">
+        <v>0</v>
+      </c>
+      <c r="O8" s="2">
+        <v>0</v>
+      </c>
+      <c r="P8" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0</v>
+      </c>
+      <c r="E9" s="2">
+        <v>0</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0</v>
+      </c>
+      <c r="H9" s="2">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2">
+        <v>0</v>
+      </c>
+      <c r="J9" s="2">
+        <v>0</v>
+      </c>
+      <c r="K9" s="2">
+        <v>0</v>
+      </c>
+      <c r="L9" s="2">
+        <v>0</v>
+      </c>
+      <c r="M9" s="2">
+        <v>0</v>
+      </c>
+      <c r="N9" s="2">
+        <v>0</v>
+      </c>
+      <c r="O9" s="2">
+        <v>0</v>
+      </c>
+      <c r="P9" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2">
+        <v>0</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2">
+        <v>0</v>
+      </c>
+      <c r="J10" s="2">
+        <v>0</v>
+      </c>
+      <c r="K10" s="2">
+        <v>0</v>
+      </c>
+      <c r="L10" s="2">
+        <v>0</v>
+      </c>
+      <c r="M10" s="2">
+        <v>0</v>
+      </c>
+      <c r="N10" s="2">
+        <v>0</v>
+      </c>
+      <c r="O10" s="2">
+        <v>0</v>
+      </c>
+      <c r="P10" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2">
+        <v>0</v>
+      </c>
+      <c r="C11" s="2">
+        <v>0</v>
+      </c>
+      <c r="D11" s="2">
+        <v>0</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2">
+        <v>0</v>
+      </c>
+      <c r="I11" s="2">
+        <v>0</v>
+      </c>
+      <c r="J11" s="2">
+        <v>0</v>
+      </c>
+      <c r="K11" s="2">
+        <v>0</v>
+      </c>
+      <c r="L11" s="2">
+        <v>0</v>
+      </c>
+      <c r="M11" s="2">
+        <v>0</v>
+      </c>
+      <c r="N11" s="2">
+        <v>0</v>
+      </c>
+      <c r="O11" s="2">
+        <v>0</v>
+      </c>
+      <c r="P11" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2">
+        <v>0</v>
+      </c>
+      <c r="C12" s="2">
+        <v>0</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0</v>
+      </c>
+      <c r="J12" s="2">
+        <v>0</v>
+      </c>
+      <c r="K12" s="2">
+        <v>0</v>
+      </c>
+      <c r="L12" s="2">
+        <v>0</v>
+      </c>
+      <c r="M12" s="2">
+        <v>0</v>
+      </c>
+      <c r="N12" s="2">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2">
+        <v>0</v>
+      </c>
+      <c r="P12" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <v>0</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0</v>
+      </c>
+      <c r="E13" s="2">
+        <v>0</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0</v>
+      </c>
+      <c r="G13" s="2">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2">
+        <v>0</v>
+      </c>
+      <c r="I13" s="2">
+        <v>0</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0</v>
+      </c>
+      <c r="K13" s="2">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2">
+        <v>0</v>
+      </c>
+      <c r="M13" s="2">
+        <v>0</v>
+      </c>
+      <c r="N13" s="2">
+        <v>0</v>
+      </c>
+      <c r="O13" s="2">
+        <v>0</v>
+      </c>
+      <c r="P13" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2">
+        <v>0</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0</v>
+      </c>
+      <c r="E14" s="2">
+        <v>0</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2">
+        <v>0</v>
+      </c>
+      <c r="H14" s="2">
+        <v>0</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0</v>
+      </c>
+      <c r="J14" s="2">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2">
+        <v>0</v>
+      </c>
+      <c r="L14" s="2">
+        <v>0</v>
+      </c>
+      <c r="M14" s="2">
+        <v>0</v>
+      </c>
+      <c r="N14" s="2">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2">
+        <v>0</v>
+      </c>
+      <c r="P14" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2">
+        <v>0</v>
+      </c>
+      <c r="C15" s="2">
+        <v>0</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2">
+        <v>0</v>
+      </c>
+      <c r="H15" s="2">
+        <v>0</v>
+      </c>
+      <c r="I15" s="2">
+        <v>0</v>
+      </c>
+      <c r="J15" s="2">
+        <v>0</v>
+      </c>
+      <c r="K15" s="2">
+        <v>0</v>
+      </c>
+      <c r="L15" s="2">
+        <v>0</v>
+      </c>
+      <c r="M15" s="2">
+        <v>0</v>
+      </c>
+      <c r="N15" s="2">
+        <v>0</v>
+      </c>
+      <c r="O15" s="2">
+        <v>0</v>
+      </c>
+      <c r="P15" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2">
+        <v>0</v>
+      </c>
+      <c r="C16" s="2">
+        <v>0</v>
+      </c>
+      <c r="D16" s="2">
+        <v>0</v>
+      </c>
+      <c r="E16" s="2">
+        <v>0</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2">
+        <v>0</v>
+      </c>
+      <c r="I16" s="2">
+        <v>0</v>
+      </c>
+      <c r="J16" s="2">
+        <v>0</v>
+      </c>
+      <c r="K16" s="2">
+        <v>0</v>
+      </c>
+      <c r="L16" s="2">
+        <v>0</v>
+      </c>
+      <c r="M16" s="2">
+        <v>0</v>
+      </c>
+      <c r="N16" s="2">
+        <v>0</v>
+      </c>
+      <c r="O16" s="2">
+        <v>0</v>
+      </c>
+      <c r="P16" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="2">
+        <v>0</v>
+      </c>
+      <c r="C17" s="2">
+        <v>0</v>
+      </c>
+      <c r="D17" s="2">
+        <v>0</v>
+      </c>
+      <c r="E17" s="2">
+        <v>0</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0</v>
+      </c>
+      <c r="H17" s="2">
+        <v>0</v>
+      </c>
+      <c r="I17" s="2">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2">
+        <v>0</v>
+      </c>
+      <c r="K17" s="2">
+        <v>0</v>
+      </c>
+      <c r="L17" s="2">
+        <v>0</v>
+      </c>
+      <c r="M17" s="2">
+        <v>0</v>
+      </c>
+      <c r="N17" s="2">
+        <v>0</v>
+      </c>
+      <c r="O17" s="2">
+        <v>0</v>
+      </c>
+      <c r="P17" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E15AAEF-9B84-E141-90CA-67AD2E5361BE}">
+  <dimension ref="A1:Q17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2">
+        <v>0</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2">
+        <v>0</v>
+      </c>
+      <c r="N2" s="2">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2">
+        <v>0</v>
+      </c>
+      <c r="P2" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C3" s="2">
+        <v>20</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2">
+        <v>0</v>
+      </c>
+      <c r="L3" s="2">
+        <v>0</v>
+      </c>
+      <c r="M3" s="2">
+        <v>0</v>
+      </c>
+      <c r="N3" s="2">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2">
+        <v>0</v>
+      </c>
+      <c r="P3" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2">
+        <v>0</v>
+      </c>
+      <c r="L4" s="2">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2">
+        <v>0</v>
+      </c>
+      <c r="N4" s="2">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2">
+        <v>0</v>
+      </c>
+      <c r="P4" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2">
+        <v>0</v>
+      </c>
+      <c r="L5" s="2">
+        <v>0</v>
+      </c>
+      <c r="M5" s="2">
+        <v>0</v>
+      </c>
+      <c r="N5" s="2">
+        <v>0</v>
+      </c>
+      <c r="O5" s="2">
+        <v>0</v>
+      </c>
+      <c r="P5" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2">
+        <v>0</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0</v>
+      </c>
+      <c r="I6" s="2">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2">
+        <v>0</v>
+      </c>
+      <c r="L6" s="2">
+        <v>0</v>
+      </c>
+      <c r="M6" s="2">
+        <v>0</v>
+      </c>
+      <c r="N6" s="2">
+        <v>0</v>
+      </c>
+      <c r="O6" s="2">
+        <v>0</v>
+      </c>
+      <c r="P6" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>0</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0</v>
+      </c>
+      <c r="J7" s="2">
+        <v>0</v>
+      </c>
+      <c r="K7" s="2">
+        <v>0</v>
+      </c>
+      <c r="L7" s="2">
+        <v>0</v>
+      </c>
+      <c r="M7" s="2">
+        <v>0</v>
+      </c>
+      <c r="N7" s="2">
+        <v>0</v>
+      </c>
+      <c r="O7" s="2">
+        <v>0</v>
+      </c>
+      <c r="P7" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <v>0</v>
+      </c>
+      <c r="C8" s="2">
+        <v>0</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2">
+        <v>0</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2">
+        <v>0</v>
+      </c>
+      <c r="J8" s="2">
+        <v>0</v>
+      </c>
+      <c r="K8" s="2">
+        <v>0</v>
+      </c>
+      <c r="L8" s="2">
+        <v>0</v>
+      </c>
+      <c r="M8" s="2">
+        <v>0</v>
+      </c>
+      <c r="N8" s="2">
+        <v>0</v>
+      </c>
+      <c r="O8" s="2">
+        <v>0</v>
+      </c>
+      <c r="P8" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0</v>
+      </c>
+      <c r="E9" s="2">
+        <v>0</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0</v>
+      </c>
+      <c r="H9" s="2">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2">
+        <v>0</v>
+      </c>
+      <c r="J9" s="2">
+        <v>0</v>
+      </c>
+      <c r="K9" s="2">
+        <v>0</v>
+      </c>
+      <c r="L9" s="2">
+        <v>0</v>
+      </c>
+      <c r="M9" s="2">
+        <v>0</v>
+      </c>
+      <c r="N9" s="2">
+        <v>0</v>
+      </c>
+      <c r="O9" s="2">
+        <v>0</v>
+      </c>
+      <c r="P9" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2">
+        <v>0</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2">
+        <v>0</v>
+      </c>
+      <c r="J10" s="2">
+        <v>0</v>
+      </c>
+      <c r="K10" s="2">
+        <v>0</v>
+      </c>
+      <c r="L10" s="2">
+        <v>0</v>
+      </c>
+      <c r="M10" s="2">
+        <v>0</v>
+      </c>
+      <c r="N10" s="2">
+        <v>0</v>
+      </c>
+      <c r="O10" s="2">
+        <v>0</v>
+      </c>
+      <c r="P10" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2">
+        <v>0</v>
+      </c>
+      <c r="C11" s="2">
+        <v>0</v>
+      </c>
+      <c r="D11" s="2">
+        <v>0</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2">
+        <v>0</v>
+      </c>
+      <c r="I11" s="2">
+        <v>0</v>
+      </c>
+      <c r="J11" s="2">
+        <v>0</v>
+      </c>
+      <c r="K11" s="2">
+        <v>0</v>
+      </c>
+      <c r="L11" s="2">
+        <v>0</v>
+      </c>
+      <c r="M11" s="2">
+        <v>0</v>
+      </c>
+      <c r="N11" s="2">
+        <v>0</v>
+      </c>
+      <c r="O11" s="2">
+        <v>0</v>
+      </c>
+      <c r="P11" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2">
+        <v>0</v>
+      </c>
+      <c r="C12" s="2">
+        <v>0</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0</v>
+      </c>
+      <c r="J12" s="2">
+        <v>0</v>
+      </c>
+      <c r="K12" s="2">
+        <v>0</v>
+      </c>
+      <c r="L12" s="2">
+        <v>0</v>
+      </c>
+      <c r="M12" s="2">
+        <v>0</v>
+      </c>
+      <c r="N12" s="2">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2">
+        <v>0</v>
+      </c>
+      <c r="P12" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <v>0</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0</v>
+      </c>
+      <c r="E13" s="2">
+        <v>0</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0</v>
+      </c>
+      <c r="G13" s="2">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2">
+        <v>0</v>
+      </c>
+      <c r="I13" s="2">
+        <v>0</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0</v>
+      </c>
+      <c r="K13" s="2">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2">
+        <v>0</v>
+      </c>
+      <c r="M13" s="2">
+        <v>0</v>
+      </c>
+      <c r="N13" s="2">
+        <v>0</v>
+      </c>
+      <c r="O13" s="2">
+        <v>0</v>
+      </c>
+      <c r="P13" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2">
+        <v>0</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0</v>
+      </c>
+      <c r="E14" s="2">
+        <v>0</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2">
+        <v>0</v>
+      </c>
+      <c r="H14" s="2">
+        <v>0</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0</v>
+      </c>
+      <c r="J14" s="2">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2">
+        <v>0</v>
+      </c>
+      <c r="L14" s="2">
+        <v>0</v>
+      </c>
+      <c r="M14" s="2">
+        <v>0</v>
+      </c>
+      <c r="N14" s="2">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2">
+        <v>0</v>
+      </c>
+      <c r="P14" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2">
+        <v>0</v>
+      </c>
+      <c r="C15" s="2">
+        <v>0</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2">
+        <v>0</v>
+      </c>
+      <c r="H15" s="2">
+        <v>0</v>
+      </c>
+      <c r="I15" s="2">
+        <v>0</v>
+      </c>
+      <c r="J15" s="2">
+        <v>0</v>
+      </c>
+      <c r="K15" s="2">
+        <v>0</v>
+      </c>
+      <c r="L15" s="2">
+        <v>0</v>
+      </c>
+      <c r="M15" s="2">
+        <v>0</v>
+      </c>
+      <c r="N15" s="2">
+        <v>0</v>
+      </c>
+      <c r="O15" s="2">
+        <v>0</v>
+      </c>
+      <c r="P15" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2">
+        <v>0</v>
+      </c>
+      <c r="C16" s="2">
+        <v>0</v>
+      </c>
+      <c r="D16" s="2">
+        <v>0</v>
+      </c>
+      <c r="E16" s="2">
+        <v>0</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2">
+        <v>0</v>
+      </c>
+      <c r="I16" s="2">
+        <v>0</v>
+      </c>
+      <c r="J16" s="2">
+        <v>0</v>
+      </c>
+      <c r="K16" s="2">
+        <v>0</v>
+      </c>
+      <c r="L16" s="2">
+        <v>0</v>
+      </c>
+      <c r="M16" s="2">
+        <v>0</v>
+      </c>
+      <c r="N16" s="2">
+        <v>0</v>
+      </c>
+      <c r="O16" s="2">
+        <v>0</v>
+      </c>
+      <c r="P16" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="2">
+        <v>0</v>
+      </c>
+      <c r="C17" s="2">
+        <v>0</v>
+      </c>
+      <c r="D17" s="2">
+        <v>0</v>
+      </c>
+      <c r="E17" s="2">
+        <v>0</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0</v>
+      </c>
+      <c r="H17" s="2">
+        <v>0</v>
+      </c>
+      <c r="I17" s="2">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2">
+        <v>0</v>
+      </c>
+      <c r="K17" s="2">
+        <v>0</v>
+      </c>
+      <c r="L17" s="2">
+        <v>0</v>
+      </c>
+      <c r="M17" s="2">
+        <v>0</v>
+      </c>
+      <c r="N17" s="2">
+        <v>0</v>
+      </c>
+      <c r="O17" s="2">
+        <v>0</v>
+      </c>
+      <c r="P17" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78B1490F-D99F-2141-A061-54CC416326CC}">
+  <dimension ref="A1:Q17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P2" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C3" s="2">
+        <v>50</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P3" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P6" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P8" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P9" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P15" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P16" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="C17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="D17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="L17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="N17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="O17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="P17" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46E51E30-728A-D044-9481-867FB0F42619}">
+  <dimension ref="A1:Q17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C3" s="2">
+        <v>50</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P6" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="H17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="L17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="M17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="N17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="O17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="P17" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>0.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add uniform mixing pool to test #223
</commit_message>
<xml_diff>
--- a/typhoidsim/data/age_mix_contact.xlsx
+++ b/typhoidsim/data/age_mix_contact.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kgrantz/active/typhoidsim/typhoidsim/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFBAEA59-984C-3E4E-9C87-B81C24A5157C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6525A32D-3329-704D-AA7E-F23CF08F8305}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="760" windowWidth="33420" windowHeight="18040" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1140" yWindow="760" windowWidth="33420" windowHeight="18040" tabRatio="500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pakistan" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="test2" sheetId="5" r:id="rId5"/>
     <sheet name="test3" sheetId="6" r:id="rId6"/>
     <sheet name="test4" sheetId="7" r:id="rId7"/>
+    <sheet name="uniform" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="20">
   <si>
     <t>age_group</t>
   </si>
@@ -7054,4 +7055,915 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D991E7B-17FF-B64A-920C-D1C8767666A5}">
+  <dimension ref="A1:Q17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2">
+        <v>1</v>
+      </c>
+      <c r="I2" s="2">
+        <v>1</v>
+      </c>
+      <c r="J2" s="2">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2">
+        <v>1</v>
+      </c>
+      <c r="L2" s="2">
+        <v>1</v>
+      </c>
+      <c r="M2" s="2">
+        <v>1</v>
+      </c>
+      <c r="N2" s="2">
+        <v>1</v>
+      </c>
+      <c r="O2" s="2">
+        <v>1</v>
+      </c>
+      <c r="P2" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2">
+        <v>1</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2">
+        <v>1</v>
+      </c>
+      <c r="J3" s="2">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2">
+        <v>1</v>
+      </c>
+      <c r="L3" s="2">
+        <v>1</v>
+      </c>
+      <c r="M3" s="2">
+        <v>1</v>
+      </c>
+      <c r="N3" s="2">
+        <v>1</v>
+      </c>
+      <c r="O3" s="2">
+        <v>1</v>
+      </c>
+      <c r="P3" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2">
+        <v>1</v>
+      </c>
+      <c r="G4" s="2">
+        <v>1</v>
+      </c>
+      <c r="H4" s="2">
+        <v>1</v>
+      </c>
+      <c r="I4" s="2">
+        <v>1</v>
+      </c>
+      <c r="J4" s="2">
+        <v>1</v>
+      </c>
+      <c r="K4" s="2">
+        <v>1</v>
+      </c>
+      <c r="L4" s="2">
+        <v>1</v>
+      </c>
+      <c r="M4" s="2">
+        <v>1</v>
+      </c>
+      <c r="N4" s="2">
+        <v>1</v>
+      </c>
+      <c r="O4" s="2">
+        <v>1</v>
+      </c>
+      <c r="P4" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2">
+        <v>1</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1</v>
+      </c>
+      <c r="G5" s="2">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2">
+        <v>1</v>
+      </c>
+      <c r="I5" s="2">
+        <v>1</v>
+      </c>
+      <c r="J5" s="2">
+        <v>1</v>
+      </c>
+      <c r="K5" s="2">
+        <v>1</v>
+      </c>
+      <c r="L5" s="2">
+        <v>1</v>
+      </c>
+      <c r="M5" s="2">
+        <v>1</v>
+      </c>
+      <c r="N5" s="2">
+        <v>1</v>
+      </c>
+      <c r="O5" s="2">
+        <v>1</v>
+      </c>
+      <c r="P5" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2">
+        <v>1</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1</v>
+      </c>
+      <c r="G6" s="2">
+        <v>1</v>
+      </c>
+      <c r="H6" s="2">
+        <v>1</v>
+      </c>
+      <c r="I6" s="2">
+        <v>1</v>
+      </c>
+      <c r="J6" s="2">
+        <v>1</v>
+      </c>
+      <c r="K6" s="2">
+        <v>1</v>
+      </c>
+      <c r="L6" s="2">
+        <v>1</v>
+      </c>
+      <c r="M6" s="2">
+        <v>1</v>
+      </c>
+      <c r="N6" s="2">
+        <v>1</v>
+      </c>
+      <c r="O6" s="2">
+        <v>1</v>
+      </c>
+      <c r="P6" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2">
+        <v>1</v>
+      </c>
+      <c r="G7" s="2">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2">
+        <v>1</v>
+      </c>
+      <c r="I7" s="2">
+        <v>1</v>
+      </c>
+      <c r="J7" s="2">
+        <v>1</v>
+      </c>
+      <c r="K7" s="2">
+        <v>1</v>
+      </c>
+      <c r="L7" s="2">
+        <v>1</v>
+      </c>
+      <c r="M7" s="2">
+        <v>1</v>
+      </c>
+      <c r="N7" s="2">
+        <v>1</v>
+      </c>
+      <c r="O7" s="2">
+        <v>1</v>
+      </c>
+      <c r="P7" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2">
+        <v>1</v>
+      </c>
+      <c r="G8" s="2">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2">
+        <v>1</v>
+      </c>
+      <c r="I8" s="2">
+        <v>1</v>
+      </c>
+      <c r="J8" s="2">
+        <v>1</v>
+      </c>
+      <c r="K8" s="2">
+        <v>1</v>
+      </c>
+      <c r="L8" s="2">
+        <v>1</v>
+      </c>
+      <c r="M8" s="2">
+        <v>1</v>
+      </c>
+      <c r="N8" s="2">
+        <v>1</v>
+      </c>
+      <c r="O8" s="2">
+        <v>1</v>
+      </c>
+      <c r="P8" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <v>1</v>
+      </c>
+      <c r="C9" s="2">
+        <v>1</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2">
+        <v>1</v>
+      </c>
+      <c r="G9" s="2">
+        <v>1</v>
+      </c>
+      <c r="H9" s="2">
+        <v>1</v>
+      </c>
+      <c r="I9" s="2">
+        <v>1</v>
+      </c>
+      <c r="J9" s="2">
+        <v>1</v>
+      </c>
+      <c r="K9" s="2">
+        <v>1</v>
+      </c>
+      <c r="L9" s="2">
+        <v>1</v>
+      </c>
+      <c r="M9" s="2">
+        <v>1</v>
+      </c>
+      <c r="N9" s="2">
+        <v>1</v>
+      </c>
+      <c r="O9" s="2">
+        <v>1</v>
+      </c>
+      <c r="P9" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2">
+        <v>1</v>
+      </c>
+      <c r="C10" s="2">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2">
+        <v>1</v>
+      </c>
+      <c r="F10" s="2">
+        <v>1</v>
+      </c>
+      <c r="G10" s="2">
+        <v>1</v>
+      </c>
+      <c r="H10" s="2">
+        <v>1</v>
+      </c>
+      <c r="I10" s="2">
+        <v>1</v>
+      </c>
+      <c r="J10" s="2">
+        <v>1</v>
+      </c>
+      <c r="K10" s="2">
+        <v>1</v>
+      </c>
+      <c r="L10" s="2">
+        <v>1</v>
+      </c>
+      <c r="M10" s="2">
+        <v>1</v>
+      </c>
+      <c r="N10" s="2">
+        <v>1</v>
+      </c>
+      <c r="O10" s="2">
+        <v>1</v>
+      </c>
+      <c r="P10" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2">
+        <v>1</v>
+      </c>
+      <c r="C11" s="2">
+        <v>1</v>
+      </c>
+      <c r="D11" s="2">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2">
+        <v>1</v>
+      </c>
+      <c r="F11" s="2">
+        <v>1</v>
+      </c>
+      <c r="G11" s="2">
+        <v>1</v>
+      </c>
+      <c r="H11" s="2">
+        <v>1</v>
+      </c>
+      <c r="I11" s="2">
+        <v>1</v>
+      </c>
+      <c r="J11" s="2">
+        <v>1</v>
+      </c>
+      <c r="K11" s="2">
+        <v>1</v>
+      </c>
+      <c r="L11" s="2">
+        <v>1</v>
+      </c>
+      <c r="M11" s="2">
+        <v>1</v>
+      </c>
+      <c r="N11" s="2">
+        <v>1</v>
+      </c>
+      <c r="O11" s="2">
+        <v>1</v>
+      </c>
+      <c r="P11" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2">
+        <v>1</v>
+      </c>
+      <c r="C12" s="2">
+        <v>1</v>
+      </c>
+      <c r="D12" s="2">
+        <v>1</v>
+      </c>
+      <c r="E12" s="2">
+        <v>1</v>
+      </c>
+      <c r="F12" s="2">
+        <v>1</v>
+      </c>
+      <c r="G12" s="2">
+        <v>1</v>
+      </c>
+      <c r="H12" s="2">
+        <v>1</v>
+      </c>
+      <c r="I12" s="2">
+        <v>1</v>
+      </c>
+      <c r="J12" s="2">
+        <v>1</v>
+      </c>
+      <c r="K12" s="2">
+        <v>1</v>
+      </c>
+      <c r="L12" s="2">
+        <v>1</v>
+      </c>
+      <c r="M12" s="2">
+        <v>1</v>
+      </c>
+      <c r="N12" s="2">
+        <v>1</v>
+      </c>
+      <c r="O12" s="2">
+        <v>1</v>
+      </c>
+      <c r="P12" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <v>1</v>
+      </c>
+      <c r="C13" s="2">
+        <v>1</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1</v>
+      </c>
+      <c r="E13" s="2">
+        <v>1</v>
+      </c>
+      <c r="F13" s="2">
+        <v>1</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1</v>
+      </c>
+      <c r="H13" s="2">
+        <v>1</v>
+      </c>
+      <c r="I13" s="2">
+        <v>1</v>
+      </c>
+      <c r="J13" s="2">
+        <v>1</v>
+      </c>
+      <c r="K13" s="2">
+        <v>1</v>
+      </c>
+      <c r="L13" s="2">
+        <v>1</v>
+      </c>
+      <c r="M13" s="2">
+        <v>1</v>
+      </c>
+      <c r="N13" s="2">
+        <v>1</v>
+      </c>
+      <c r="O13" s="2">
+        <v>1</v>
+      </c>
+      <c r="P13" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2">
+        <v>1</v>
+      </c>
+      <c r="C14" s="2">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2">
+        <v>1</v>
+      </c>
+      <c r="E14" s="2">
+        <v>1</v>
+      </c>
+      <c r="F14" s="2">
+        <v>1</v>
+      </c>
+      <c r="G14" s="2">
+        <v>1</v>
+      </c>
+      <c r="H14" s="2">
+        <v>1</v>
+      </c>
+      <c r="I14" s="2">
+        <v>1</v>
+      </c>
+      <c r="J14" s="2">
+        <v>1</v>
+      </c>
+      <c r="K14" s="2">
+        <v>1</v>
+      </c>
+      <c r="L14" s="2">
+        <v>1</v>
+      </c>
+      <c r="M14" s="2">
+        <v>1</v>
+      </c>
+      <c r="N14" s="2">
+        <v>1</v>
+      </c>
+      <c r="O14" s="2">
+        <v>1</v>
+      </c>
+      <c r="P14" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2">
+        <v>1</v>
+      </c>
+      <c r="C15" s="2">
+        <v>1</v>
+      </c>
+      <c r="D15" s="2">
+        <v>1</v>
+      </c>
+      <c r="E15" s="2">
+        <v>1</v>
+      </c>
+      <c r="F15" s="2">
+        <v>1</v>
+      </c>
+      <c r="G15" s="2">
+        <v>1</v>
+      </c>
+      <c r="H15" s="2">
+        <v>1</v>
+      </c>
+      <c r="I15" s="2">
+        <v>1</v>
+      </c>
+      <c r="J15" s="2">
+        <v>1</v>
+      </c>
+      <c r="K15" s="2">
+        <v>1</v>
+      </c>
+      <c r="L15" s="2">
+        <v>1</v>
+      </c>
+      <c r="M15" s="2">
+        <v>1</v>
+      </c>
+      <c r="N15" s="2">
+        <v>1</v>
+      </c>
+      <c r="O15" s="2">
+        <v>1</v>
+      </c>
+      <c r="P15" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2">
+        <v>1</v>
+      </c>
+      <c r="C16" s="2">
+        <v>1</v>
+      </c>
+      <c r="D16" s="2">
+        <v>1</v>
+      </c>
+      <c r="E16" s="2">
+        <v>1</v>
+      </c>
+      <c r="F16" s="2">
+        <v>1</v>
+      </c>
+      <c r="G16" s="2">
+        <v>1</v>
+      </c>
+      <c r="H16" s="2">
+        <v>1</v>
+      </c>
+      <c r="I16" s="2">
+        <v>1</v>
+      </c>
+      <c r="J16" s="2">
+        <v>1</v>
+      </c>
+      <c r="K16" s="2">
+        <v>1</v>
+      </c>
+      <c r="L16" s="2">
+        <v>1</v>
+      </c>
+      <c r="M16" s="2">
+        <v>1</v>
+      </c>
+      <c r="N16" s="2">
+        <v>1</v>
+      </c>
+      <c r="O16" s="2">
+        <v>1</v>
+      </c>
+      <c r="P16" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="2">
+        <v>1</v>
+      </c>
+      <c r="C17" s="2">
+        <v>1</v>
+      </c>
+      <c r="D17" s="2">
+        <v>1</v>
+      </c>
+      <c r="E17" s="2">
+        <v>1</v>
+      </c>
+      <c r="F17" s="2">
+        <v>1</v>
+      </c>
+      <c r="G17" s="2">
+        <v>1</v>
+      </c>
+      <c r="H17" s="2">
+        <v>1</v>
+      </c>
+      <c r="I17" s="2">
+        <v>1</v>
+      </c>
+      <c r="J17" s="2">
+        <v>1</v>
+      </c>
+      <c r="K17" s="2">
+        <v>1</v>
+      </c>
+      <c r="L17" s="2">
+        <v>1</v>
+      </c>
+      <c r="M17" s="2">
+        <v>1</v>
+      </c>
+      <c r="N17" s="2">
+        <v>1</v>
+      </c>
+      <c r="O17" s="2">
+        <v>1</v>
+      </c>
+      <c r="P17" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>